<commit_message>
fix mistakes, update coremark/Mhz
</commit_message>
<xml_diff>
--- a/CoreMark/CoreMark.xlsx
+++ b/CoreMark/CoreMark.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\archive\github\benchmark\CoreMark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1436DA8-C66D-41A0-A8DE-4BEEFEAB1B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8E86F2-602A-402C-82E3-A61A35A0F4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29025" yWindow="255" windowWidth="21150" windowHeight="15030" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29670" yWindow="105" windowWidth="26505" windowHeight="15705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="2025" sheetId="3" r:id="rId1"/>
-    <sheet name="multi" sheetId="2" r:id="rId2"/>
-    <sheet name="single2021" sheetId="1" r:id="rId3"/>
+    <sheet name="2026" sheetId="4" r:id="rId1"/>
+    <sheet name="2025" sheetId="3" r:id="rId2"/>
+    <sheet name="multi" sheetId="2" r:id="rId3"/>
+    <sheet name="single2021" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="112">
   <si>
     <t>CoreMark Values</t>
   </si>
@@ -342,6 +346,33 @@
   </si>
   <si>
     <t>theory</t>
+  </si>
+  <si>
+    <t>Galaxy Note 20</t>
+  </si>
+  <si>
+    <t>Snapdragpon 865</t>
+  </si>
+  <si>
+    <t>ARMv8.2-A</t>
+  </si>
+  <si>
+    <t>NEW</t>
+  </si>
+  <si>
+    <t>Galaxy S24</t>
+  </si>
+  <si>
+    <t>ARMv9.2-A</t>
+  </si>
+  <si>
+    <t>Cortex-X4 </t>
+  </si>
+  <si>
+    <t>Exynos 2400</t>
+  </si>
+  <si>
+    <t>Kyro 585</t>
   </si>
 </sst>
 </file>
@@ -373,7 +404,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -395,6 +426,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF7C80"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -432,7 +469,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -460,10 +497,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Link" xfId="1" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -484,7 +522,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -778,10 +816,58 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="0" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{52DDD5D5-7268-427D-A1A4-19C1D3E709F7}">
+  <we:reference id="wa200005502" version="1.0.0.12" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200005502" version="1.0.0.12" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_GPT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_CREATE_PROMPT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_LIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_HLIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_CLASSIFY</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_TRANSLATE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_EXTRACT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_TAG</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_CONVERT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_FORMAT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_SUMMARIZE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_TABLE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_FILL</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_SPLIT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_HSPLIT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_EDIT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_MATCH</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_VISION</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_WEB</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9321212E-8ABB-4B14-AEF6-E9EC57B10669}">
-  <dimension ref="A1:P31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D838E1AF-0657-4DA5-A1B8-069399C72A73}">
+  <dimension ref="A1:P33"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
@@ -882,6 +968,1092 @@
       <c r="J4" s="14">
         <v>1997</v>
       </c>
+      <c r="K4" s="11">
+        <f>C4/D4</f>
+        <v>0.4375</v>
+      </c>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="14">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1">
+        <f t="shared" ref="B5:B19" si="0">C5/D5</f>
+        <v>1.125</v>
+      </c>
+      <c r="C5">
+        <v>81</v>
+      </c>
+      <c r="D5">
+        <v>72</v>
+      </c>
+      <c r="F5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5">
+        <v>32</v>
+      </c>
+      <c r="J5">
+        <v>2007</v>
+      </c>
+      <c r="K5" s="11">
+        <f>C5/D5</f>
+        <v>1.125</v>
+      </c>
+      <c r="O5">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="1">
+        <f t="shared" si="0"/>
+        <v>1.7857142857142858</v>
+      </c>
+      <c r="C6">
+        <v>150</v>
+      </c>
+      <c r="D6">
+        <v>84</v>
+      </c>
+      <c r="F6" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6">
+        <v>32</v>
+      </c>
+      <c r="J6">
+        <v>2013</v>
+      </c>
+      <c r="K6" s="1">
+        <f t="shared" ref="K6:K14" si="1">C6/D6</f>
+        <v>1.7857142857142858</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="O6">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="1">
+        <f t="shared" si="0"/>
+        <v>1.72</v>
+      </c>
+      <c r="C7">
+        <v>172</v>
+      </c>
+      <c r="D7">
+        <v>100</v>
+      </c>
+      <c r="F7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7">
+        <v>32</v>
+      </c>
+      <c r="J7">
+        <v>2013</v>
+      </c>
+      <c r="K7" s="1">
+        <f t="shared" si="1"/>
+        <v>1.72</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="O7">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="1">
+        <f t="shared" si="0"/>
+        <v>1.481203007518797</v>
+      </c>
+      <c r="C8">
+        <v>197</v>
+      </c>
+      <c r="D8">
+        <v>133</v>
+      </c>
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8">
+        <v>32</v>
+      </c>
+      <c r="J8">
+        <v>2021</v>
+      </c>
+      <c r="K8" s="1">
+        <f t="shared" si="1"/>
+        <v>1.481203007518797</v>
+      </c>
+      <c r="N8" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="O8" s="3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="1">
+        <f t="shared" si="0"/>
+        <v>1.9</v>
+      </c>
+      <c r="C9">
+        <v>304</v>
+      </c>
+      <c r="D9">
+        <v>160</v>
+      </c>
+      <c r="E9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" t="s">
+        <v>86</v>
+      </c>
+      <c r="G9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9">
+        <v>32</v>
+      </c>
+      <c r="J9">
+        <v>2016</v>
+      </c>
+      <c r="K9" s="1">
+        <f t="shared" si="1"/>
+        <v>1.9</v>
+      </c>
+      <c r="M9" t="s">
+        <v>87</v>
+      </c>
+      <c r="O9" s="3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1">
+        <f t="shared" si="0"/>
+        <v>2.1937500000000001</v>
+      </c>
+      <c r="C10">
+        <v>351</v>
+      </c>
+      <c r="D10">
+        <v>160</v>
+      </c>
+      <c r="F10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" t="s">
+        <v>80</v>
+      </c>
+      <c r="H10">
+        <v>32</v>
+      </c>
+      <c r="J10">
+        <v>2016</v>
+      </c>
+      <c r="K10" s="1">
+        <f t="shared" si="1"/>
+        <v>2.1937500000000001</v>
+      </c>
+      <c r="N10" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="O10">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="1">
+        <f t="shared" si="0"/>
+        <v>2.2562500000000001</v>
+      </c>
+      <c r="C11">
+        <v>361</v>
+      </c>
+      <c r="D11">
+        <v>160</v>
+      </c>
+      <c r="F11" t="s">
+        <v>81</v>
+      </c>
+      <c r="G11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H11">
+        <v>32</v>
+      </c>
+      <c r="J11">
+        <v>2019</v>
+      </c>
+      <c r="K11" s="1">
+        <f t="shared" si="1"/>
+        <v>2.2562500000000001</v>
+      </c>
+      <c r="N11" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="O11" s="3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="1">
+        <f t="shared" si="0"/>
+        <v>2.34375</v>
+      </c>
+      <c r="C12">
+        <v>375</v>
+      </c>
+      <c r="D12">
+        <v>160</v>
+      </c>
+      <c r="F12" t="s">
+        <v>81</v>
+      </c>
+      <c r="G12" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12">
+        <v>32</v>
+      </c>
+      <c r="J12">
+        <v>2016</v>
+      </c>
+      <c r="K12" s="1">
+        <f t="shared" si="1"/>
+        <v>2.34375</v>
+      </c>
+      <c r="N12" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="O12" s="3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="1">
+        <f t="shared" si="0"/>
+        <v>1.8791666666666667</v>
+      </c>
+      <c r="C13">
+        <v>451</v>
+      </c>
+      <c r="D13">
+        <v>240</v>
+      </c>
+      <c r="F13" t="s">
+        <v>81</v>
+      </c>
+      <c r="G13" t="s">
+        <v>79</v>
+      </c>
+      <c r="H13">
+        <v>32</v>
+      </c>
+      <c r="J13">
+        <v>2020</v>
+      </c>
+      <c r="K13" s="1">
+        <f t="shared" si="1"/>
+        <v>1.8791666666666667</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="N13" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="O13" s="3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="1">
+        <f t="shared" si="0"/>
+        <v>2.2485714285714287</v>
+      </c>
+      <c r="C14">
+        <v>1574</v>
+      </c>
+      <c r="D14">
+        <v>700</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14">
+        <v>32</v>
+      </c>
+      <c r="J14">
+        <v>2012</v>
+      </c>
+      <c r="K14" s="1">
+        <f t="shared" si="1"/>
+        <v>2.2485714285714287</v>
+      </c>
+      <c r="N14" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="O14">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="1">
+        <f t="shared" si="0"/>
+        <v>2.8436154949784793</v>
+      </c>
+      <c r="C15">
+        <v>3964</v>
+      </c>
+      <c r="D15">
+        <v>1394</v>
+      </c>
+      <c r="E15" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" t="s">
+        <v>89</v>
+      </c>
+      <c r="H15">
+        <v>32</v>
+      </c>
+      <c r="J15">
+        <v>2018</v>
+      </c>
+      <c r="K15" s="1">
+        <f>C15/D15</f>
+        <v>2.8436154949784793</v>
+      </c>
+      <c r="N15" s="6">
+        <v>1</v>
+      </c>
+      <c r="O15" s="3">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="11">
+        <f t="shared" si="0"/>
+        <v>3.1666666666666665</v>
+      </c>
+      <c r="C16" s="12">
+        <v>3800</v>
+      </c>
+      <c r="D16" s="12">
+        <v>1200</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="H16" s="12">
+        <v>64</v>
+      </c>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12">
+        <v>2016</v>
+      </c>
+      <c r="K16" s="11">
+        <f>C16/D16</f>
+        <v>3.1666666666666665</v>
+      </c>
+      <c r="L16" s="12"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="13">
+        <v>1</v>
+      </c>
+      <c r="O16" s="12">
+        <v>2020</v>
+      </c>
+      <c r="P16" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="1">
+        <f t="shared" si="0"/>
+        <v>3.2608333333333333</v>
+      </c>
+      <c r="C17">
+        <v>3913</v>
+      </c>
+      <c r="D17">
+        <v>1200</v>
+      </c>
+      <c r="E17" t="s">
+        <v>95</v>
+      </c>
+      <c r="F17" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17" t="s">
+        <v>61</v>
+      </c>
+      <c r="H17">
+        <v>64</v>
+      </c>
+      <c r="J17">
+        <v>2015</v>
+      </c>
+      <c r="K17" s="1">
+        <f t="shared" ref="K17:K21" si="2">C17/D17</f>
+        <v>3.2608333333333333</v>
+      </c>
+      <c r="O17">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="1">
+        <f t="shared" si="0"/>
+        <v>5.504666666666667</v>
+      </c>
+      <c r="C18">
+        <v>8257</v>
+      </c>
+      <c r="D18">
+        <v>1500</v>
+      </c>
+      <c r="E18" t="s">
+        <v>94</v>
+      </c>
+      <c r="F18" t="s">
+        <v>63</v>
+      </c>
+      <c r="G18" t="s">
+        <v>93</v>
+      </c>
+      <c r="H18">
+        <v>64</v>
+      </c>
+      <c r="J18">
+        <v>2019</v>
+      </c>
+      <c r="K18" s="1">
+        <f t="shared" si="2"/>
+        <v>5.504666666666667</v>
+      </c>
+      <c r="N18" s="6">
+        <v>4</v>
+      </c>
+      <c r="O18">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="1">
+        <f t="shared" si="0"/>
+        <v>4.4584967320261439</v>
+      </c>
+      <c r="C19">
+        <v>13643</v>
+      </c>
+      <c r="D19">
+        <v>3060</v>
+      </c>
+      <c r="E19" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" t="s">
+        <v>64</v>
+      </c>
+      <c r="G19" t="s">
+        <v>65</v>
+      </c>
+      <c r="H19">
+        <v>64</v>
+      </c>
+      <c r="I19">
+        <v>45</v>
+      </c>
+      <c r="J19">
+        <v>2009</v>
+      </c>
+      <c r="K19" s="1">
+        <f t="shared" si="2"/>
+        <v>4.4584967320261439</v>
+      </c>
+      <c r="N19" s="6">
+        <v>24</v>
+      </c>
+      <c r="O19">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="1">
+        <f>C20/D20</f>
+        <v>6.3620000000000001</v>
+      </c>
+      <c r="C20">
+        <v>19086</v>
+      </c>
+      <c r="D20">
+        <v>3000</v>
+      </c>
+      <c r="E20" t="s">
+        <v>82</v>
+      </c>
+      <c r="F20" t="s">
+        <v>64</v>
+      </c>
+      <c r="G20" t="s">
+        <v>66</v>
+      </c>
+      <c r="H20">
+        <v>64</v>
+      </c>
+      <c r="I20">
+        <v>22</v>
+      </c>
+      <c r="J20">
+        <v>2013</v>
+      </c>
+      <c r="K20" s="1">
+        <f t="shared" si="2"/>
+        <v>6.3620000000000001</v>
+      </c>
+      <c r="N20" s="6">
+        <v>16</v>
+      </c>
+      <c r="O20">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="1">
+        <f t="shared" ref="B21:B27" si="3">C21/D21</f>
+        <v>6.4378787878787875</v>
+      </c>
+      <c r="C21">
+        <v>21245</v>
+      </c>
+      <c r="D21">
+        <v>3300</v>
+      </c>
+      <c r="E21" t="s">
+        <v>82</v>
+      </c>
+      <c r="F21" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" t="s">
+        <v>66</v>
+      </c>
+      <c r="H21">
+        <v>64</v>
+      </c>
+      <c r="I21">
+        <v>22</v>
+      </c>
+      <c r="J21">
+        <v>2012</v>
+      </c>
+      <c r="K21" s="1">
+        <f t="shared" si="2"/>
+        <v>6.4378787878787875</v>
+      </c>
+      <c r="N21" s="6">
+        <v>16</v>
+      </c>
+      <c r="O21">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="1">
+        <f t="shared" si="3"/>
+        <v>6.4969945355191259</v>
+      </c>
+      <c r="C22">
+        <v>23779</v>
+      </c>
+      <c r="D22">
+        <v>3660</v>
+      </c>
+      <c r="E22" t="s">
+        <v>84</v>
+      </c>
+      <c r="F22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" t="s">
+        <v>67</v>
+      </c>
+      <c r="H22">
+        <v>64</v>
+      </c>
+      <c r="I22">
+        <v>14</v>
+      </c>
+      <c r="J22">
+        <v>2015</v>
+      </c>
+      <c r="K22" s="1">
+        <f>C22/D22</f>
+        <v>6.4969945355191259</v>
+      </c>
+      <c r="N22" s="6">
+        <v>24</v>
+      </c>
+      <c r="O22">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="1">
+        <f t="shared" si="3"/>
+        <v>7.2350710900473931</v>
+      </c>
+      <c r="C23">
+        <v>30532</v>
+      </c>
+      <c r="D23">
+        <v>4220</v>
+      </c>
+      <c r="E23" t="s">
+        <v>85</v>
+      </c>
+      <c r="F23" t="s">
+        <v>64</v>
+      </c>
+      <c r="G23" t="s">
+        <v>68</v>
+      </c>
+      <c r="H23">
+        <v>64</v>
+      </c>
+      <c r="I23">
+        <v>14</v>
+      </c>
+      <c r="J23">
+        <v>2020</v>
+      </c>
+      <c r="K23" s="1">
+        <f>C23/D23</f>
+        <v>7.2350710900473931</v>
+      </c>
+      <c r="N23" s="6">
+        <v>48</v>
+      </c>
+      <c r="O23">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" s="1">
+        <f>C24/D24</f>
+        <v>7.6503125000000001</v>
+      </c>
+      <c r="C24">
+        <v>24481</v>
+      </c>
+      <c r="D24">
+        <v>3200</v>
+      </c>
+      <c r="E24" t="s">
+        <v>104</v>
+      </c>
+      <c r="F24" t="s">
+        <v>105</v>
+      </c>
+      <c r="G24" t="s">
+        <v>111</v>
+      </c>
+      <c r="H24">
+        <v>64</v>
+      </c>
+      <c r="I24">
+        <v>7</v>
+      </c>
+      <c r="J24">
+        <v>2020</v>
+      </c>
+      <c r="K24" s="1">
+        <f>C24/D24</f>
+        <v>7.6503125000000001</v>
+      </c>
+      <c r="N24" s="6">
+        <v>8</v>
+      </c>
+      <c r="O24" s="3">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="1">
+        <f t="shared" si="3"/>
+        <v>8.4960869565217383</v>
+      </c>
+      <c r="C25">
+        <v>39082</v>
+      </c>
+      <c r="D25">
+        <v>4600</v>
+      </c>
+      <c r="E25" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" t="s">
+        <v>64</v>
+      </c>
+      <c r="G25" t="s">
+        <v>75</v>
+      </c>
+      <c r="H25">
+        <v>64</v>
+      </c>
+      <c r="I25">
+        <v>7</v>
+      </c>
+      <c r="J25">
+        <v>2023</v>
+      </c>
+      <c r="K25" s="1">
+        <f>C25/D25</f>
+        <v>8.4960869565217383</v>
+      </c>
+      <c r="N25" s="6">
+        <v>64</v>
+      </c>
+      <c r="O25">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>43</v>
+      </c>
+      <c r="B26" s="1">
+        <f t="shared" ref="B26" si="4">C26/D26</f>
+        <v>9.9118750000000002</v>
+      </c>
+      <c r="C26">
+        <v>31718</v>
+      </c>
+      <c r="D26">
+        <v>3200</v>
+      </c>
+      <c r="E26" t="s">
+        <v>72</v>
+      </c>
+      <c r="F26" t="s">
+        <v>71</v>
+      </c>
+      <c r="G26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H26">
+        <v>64</v>
+      </c>
+      <c r="I26">
+        <v>5</v>
+      </c>
+      <c r="J26">
+        <v>2020</v>
+      </c>
+      <c r="K26" s="1">
+        <f>C26/D26</f>
+        <v>9.9118750000000002</v>
+      </c>
+      <c r="N26" s="6">
+        <v>16</v>
+      </c>
+      <c r="O26" s="3">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B27" s="1">
+        <f t="shared" si="3"/>
+        <v>10.320560747663551</v>
+      </c>
+      <c r="C27">
+        <v>33129</v>
+      </c>
+      <c r="D27">
+        <v>3210</v>
+      </c>
+      <c r="E27" t="s">
+        <v>110</v>
+      </c>
+      <c r="F27" t="s">
+        <v>108</v>
+      </c>
+      <c r="G27" t="s">
+        <v>109</v>
+      </c>
+      <c r="H27">
+        <v>64</v>
+      </c>
+      <c r="I27">
+        <v>4</v>
+      </c>
+      <c r="J27">
+        <v>2024</v>
+      </c>
+      <c r="K27" s="1">
+        <f>C27/D27</f>
+        <v>10.320560747663551</v>
+      </c>
+      <c r="M27" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="N27" s="6">
+        <v>8</v>
+      </c>
+      <c r="O27" s="3">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="B29" s="1">
+        <f>C29/D29</f>
+        <v>10.320560747663551</v>
+      </c>
+      <c r="C29">
+        <v>33129</v>
+      </c>
+      <c r="D29">
+        <v>3210</v>
+      </c>
+      <c r="K29" s="1">
+        <f>C29/D29</f>
+        <v>10.320560747663551</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="F33" t="s">
+        <v>98</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A33" r:id="rId1" xr:uid="{1533EFA7-4865-4211-9D32-F2745D021C3D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9321212E-8ABB-4B14-AEF6-E9EC57B10669}">
+  <dimension ref="A1:P31"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="4.42578125" customWidth="1"/>
+    <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" customWidth="1"/>
+    <col min="14" max="14" width="5.140625" style="6" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N2" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="15">
+        <f>C4/D4</f>
+        <v>0.4375</v>
+      </c>
+      <c r="C4" s="14">
+        <v>7</v>
+      </c>
+      <c r="D4" s="14">
+        <v>16</v>
+      </c>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="H4" s="14">
+        <v>8</v>
+      </c>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14">
+        <v>1997</v>
+      </c>
       <c r="K4" s="14"/>
       <c r="L4" s="14"/>
       <c r="M4" s="14"/>
@@ -1649,10 +2821,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{978EF068-C664-40CD-A690-2ADA683B78C9}">
   <dimension ref="A1:D31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -1934,10 +3106,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
include Archer C7 for CoreMark
</commit_message>
<xml_diff>
--- a/CoreMark/CoreMark.xlsx
+++ b/CoreMark/CoreMark.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\archive\github\benchmark\CoreMark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8E86F2-602A-402C-82E3-A61A35A0F4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11653733-D395-4442-A518-D3FFA44B9818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29670" yWindow="105" windowWidth="26505" windowHeight="15705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6795" yWindow="1395" windowWidth="19995" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="116">
   <si>
     <t>CoreMark Values</t>
   </si>
@@ -373,6 +373,18 @@
   </si>
   <si>
     <t>Kyro 585</t>
+  </si>
+  <si>
+    <t>Qualcomm Atheros QCA956X</t>
+  </si>
+  <si>
+    <t>TP-Link Archer C7</t>
+  </si>
+  <si>
+    <t>QCA956X</t>
+  </si>
+  <si>
+    <t>MIPS 74Kc V5.0</t>
   </si>
 </sst>
 </file>
@@ -404,7 +416,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -432,6 +444,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -469,7 +487,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -498,6 +516,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -866,7 +886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D838E1AF-0657-4DA5-A1B8-069399C72A73}">
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -883,17 +903,17 @@
     <col min="14" max="14" width="5.140625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="N2" s="6" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
@@ -940,7 +960,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>5</v>
       </c>
@@ -979,12 +999,12 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1">
-        <f t="shared" ref="B5:B19" si="0">C5/D5</f>
+        <f t="shared" ref="B5:B20" si="0">C5/D5</f>
         <v>1.125</v>
       </c>
       <c r="C5">
@@ -999,7 +1019,7 @@
       <c r="G5" t="s">
         <v>49</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="19">
         <v>32</v>
       </c>
       <c r="J5">
@@ -1013,7 +1033,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1033,14 +1053,14 @@
       <c r="G6" t="s">
         <v>52</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="19">
         <v>32</v>
       </c>
       <c r="J6">
         <v>2013</v>
       </c>
       <c r="K6" s="1">
-        <f t="shared" ref="K6:K14" si="1">C6/D6</f>
+        <f t="shared" ref="K6:K15" si="1">C6/D6</f>
         <v>1.7857142857142858</v>
       </c>
       <c r="M6" s="4" t="s">
@@ -1050,7 +1070,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1070,7 +1090,7 @@
       <c r="G7" t="s">
         <v>52</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="19">
         <v>32</v>
       </c>
       <c r="J7">
@@ -1087,7 +1107,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>37</v>
       </c>
@@ -1110,7 +1130,7 @@
       <c r="G8" t="s">
         <v>55</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="19">
         <v>32</v>
       </c>
       <c r="J8">
@@ -1127,7 +1147,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>42</v>
       </c>
@@ -1150,7 +1170,7 @@
       <c r="G9" t="s">
         <v>47</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="19">
         <v>32</v>
       </c>
       <c r="J9">
@@ -1167,7 +1187,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1187,7 +1207,7 @@
       <c r="G10" t="s">
         <v>80</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="19">
         <v>32</v>
       </c>
       <c r="J10">
@@ -1204,7 +1224,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1224,7 +1244,7 @@
       <c r="G11" t="s">
         <v>79</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="19">
         <v>32</v>
       </c>
       <c r="J11">
@@ -1241,7 +1261,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -1261,7 +1281,7 @@
       <c r="G12" t="s">
         <v>80</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="19">
         <v>32</v>
       </c>
       <c r="J12">
@@ -1278,7 +1298,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -1298,7 +1318,7 @@
       <c r="G13" t="s">
         <v>79</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="19">
         <v>32</v>
       </c>
       <c r="J13">
@@ -1318,7 +1338,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>10</v>
       </c>
@@ -1338,7 +1358,7 @@
       <c r="G14" t="s">
         <v>59</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="19">
         <v>32</v>
       </c>
       <c r="J14">
@@ -1355,595 +1375,631 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B15" s="1">
+        <v>2.65</v>
+      </c>
+      <c r="C15">
+        <v>2053</v>
+      </c>
+      <c r="D15">
+        <v>775</v>
+      </c>
+      <c r="E15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F15" t="s">
+        <v>115</v>
+      </c>
+      <c r="G15" t="s">
+        <v>114</v>
+      </c>
+      <c r="H15" s="19">
+        <v>32</v>
+      </c>
+      <c r="J15">
+        <v>2011</v>
+      </c>
+      <c r="K15" s="1">
+        <f t="shared" si="1"/>
+        <v>2.649032258064516</v>
+      </c>
+      <c r="O15" s="3">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B16" s="1">
         <f t="shared" si="0"/>
         <v>2.8436154949784793</v>
       </c>
-      <c r="C15">
+      <c r="C16">
         <v>3964</v>
       </c>
-      <c r="D15">
+      <c r="D16">
         <v>1394</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E16" t="s">
         <v>90</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F16" t="s">
         <v>92</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G16" t="s">
         <v>89</v>
       </c>
-      <c r="H15">
+      <c r="H16" s="19">
         <v>32</v>
       </c>
-      <c r="J15">
+      <c r="J16">
         <v>2018</v>
       </c>
-      <c r="K15" s="1">
-        <f>C15/D15</f>
+      <c r="K16" s="1">
+        <f>C16/D16</f>
         <v>2.8436154949784793</v>
       </c>
-      <c r="N15" s="6">
+      <c r="N16" s="6">
         <v>1</v>
       </c>
-      <c r="O15" s="3">
+      <c r="O16" s="3">
         <v>2025</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B17" s="11">
         <f t="shared" si="0"/>
         <v>3.1666666666666665</v>
       </c>
-      <c r="C16" s="12">
+      <c r="C17" s="12">
         <v>3800</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D17" s="12">
         <v>1200</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E17" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F17" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="G16" s="12" t="s">
+      <c r="G17" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H16" s="12">
-        <v>64</v>
-      </c>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12">
+      <c r="H17" s="12">
+        <v>64</v>
+      </c>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12">
         <v>2016</v>
       </c>
-      <c r="K16" s="11">
-        <f>C16/D16</f>
+      <c r="K17" s="11">
+        <f>C17/D17</f>
         <v>3.1666666666666665</v>
       </c>
-      <c r="L16" s="12"/>
-      <c r="M16" s="12"/>
-      <c r="N16" s="13">
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="13">
         <v>1</v>
       </c>
-      <c r="O16" s="12">
+      <c r="O17" s="12">
         <v>2020</v>
       </c>
-      <c r="P16" t="s">
+      <c r="P17" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B18" s="1">
         <f t="shared" si="0"/>
         <v>3.2608333333333333</v>
       </c>
-      <c r="C17">
+      <c r="C18">
         <v>3913</v>
       </c>
-      <c r="D17">
+      <c r="D18">
         <v>1200</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E18" t="s">
         <v>95</v>
-      </c>
-      <c r="F17" t="s">
-        <v>63</v>
-      </c>
-      <c r="G17" t="s">
-        <v>61</v>
-      </c>
-      <c r="H17">
-        <v>64</v>
-      </c>
-      <c r="J17">
-        <v>2015</v>
-      </c>
-      <c r="K17" s="1">
-        <f t="shared" ref="K17:K21" si="2">C17/D17</f>
-        <v>3.2608333333333333</v>
-      </c>
-      <c r="O17">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B18" s="1">
-        <f t="shared" si="0"/>
-        <v>5.504666666666667</v>
-      </c>
-      <c r="C18">
-        <v>8257</v>
-      </c>
-      <c r="D18">
-        <v>1500</v>
-      </c>
-      <c r="E18" t="s">
-        <v>94</v>
       </c>
       <c r="F18" t="s">
         <v>63</v>
       </c>
       <c r="G18" t="s">
+        <v>61</v>
+      </c>
+      <c r="H18">
+        <v>64</v>
+      </c>
+      <c r="J18">
+        <v>2015</v>
+      </c>
+      <c r="K18" s="1">
+        <f t="shared" ref="K18:K22" si="2">C18/D18</f>
+        <v>3.2608333333333333</v>
+      </c>
+      <c r="O18">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B19" s="1">
+        <f t="shared" si="0"/>
+        <v>5.504666666666667</v>
+      </c>
+      <c r="C19">
+        <v>8257</v>
+      </c>
+      <c r="D19">
+        <v>1500</v>
+      </c>
+      <c r="E19" t="s">
+        <v>94</v>
+      </c>
+      <c r="F19" t="s">
+        <v>63</v>
+      </c>
+      <c r="G19" t="s">
         <v>93</v>
       </c>
-      <c r="H18">
-        <v>64</v>
-      </c>
-      <c r="J18">
+      <c r="H19">
+        <v>64</v>
+      </c>
+      <c r="J19">
         <v>2019</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K19" s="1">
         <f t="shared" si="2"/>
         <v>5.504666666666667</v>
       </c>
-      <c r="N18" s="6">
+      <c r="N19" s="6">
         <v>4</v>
       </c>
-      <c r="O18">
+      <c r="O19">
         <v>2025</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B20" s="1">
         <f t="shared" si="0"/>
         <v>4.4584967320261439</v>
       </c>
-      <c r="C19">
+      <c r="C20">
         <v>13643</v>
       </c>
-      <c r="D19">
+      <c r="D20">
         <v>3060</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E20" t="s">
         <v>83</v>
       </c>
-      <c r="F19" t="s">
-        <v>64</v>
-      </c>
-      <c r="G19" t="s">
+      <c r="F20" t="s">
+        <v>64</v>
+      </c>
+      <c r="G20" t="s">
         <v>65</v>
       </c>
-      <c r="H19">
-        <v>64</v>
-      </c>
-      <c r="I19">
+      <c r="H20">
+        <v>64</v>
+      </c>
+      <c r="I20">
         <v>45</v>
       </c>
-      <c r="J19">
+      <c r="J20">
         <v>2009</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K20" s="1">
         <f t="shared" si="2"/>
         <v>4.4584967320261439</v>
       </c>
-      <c r="N19" s="6">
+      <c r="N20" s="6">
         <v>24</v>
       </c>
-      <c r="O19">
+      <c r="O20">
         <v>2020</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>76</v>
       </c>
-      <c r="B20" s="1">
-        <f>C20/D20</f>
+      <c r="B21" s="1">
+        <f>C21/D21</f>
         <v>6.3620000000000001</v>
       </c>
-      <c r="C20">
+      <c r="C21">
         <v>19086</v>
       </c>
-      <c r="D20">
+      <c r="D21">
         <v>3000</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E21" t="s">
         <v>82</v>
       </c>
-      <c r="F20" t="s">
-        <v>64</v>
-      </c>
-      <c r="G20" t="s">
+      <c r="F21" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" t="s">
         <v>66</v>
       </c>
-      <c r="H20">
-        <v>64</v>
-      </c>
-      <c r="I20">
+      <c r="H21">
+        <v>64</v>
+      </c>
+      <c r="I21">
         <v>22</v>
       </c>
-      <c r="J20">
+      <c r="J21">
         <v>2013</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K21" s="1">
         <f t="shared" si="2"/>
         <v>6.3620000000000001</v>
       </c>
-      <c r="N20" s="6">
+      <c r="N21" s="6">
         <v>16</v>
       </c>
-      <c r="O20">
+      <c r="O21">
         <v>2024</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="1">
-        <f t="shared" ref="B21:B27" si="3">C21/D21</f>
+      <c r="B22" s="1">
+        <f t="shared" ref="B22:B28" si="3">C22/D22</f>
         <v>6.4378787878787875</v>
       </c>
-      <c r="C21">
+      <c r="C22">
         <v>21245</v>
       </c>
-      <c r="D21">
+      <c r="D22">
         <v>3300</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E22" t="s">
         <v>82</v>
       </c>
-      <c r="F21" t="s">
-        <v>64</v>
-      </c>
-      <c r="G21" t="s">
+      <c r="F22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" t="s">
         <v>66</v>
       </c>
-      <c r="H21">
-        <v>64</v>
-      </c>
-      <c r="I21">
+      <c r="H22">
+        <v>64</v>
+      </c>
+      <c r="I22">
         <v>22</v>
       </c>
-      <c r="J21">
+      <c r="J22">
         <v>2012</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K22" s="1">
         <f t="shared" si="2"/>
         <v>6.4378787878787875</v>
       </c>
-      <c r="N21" s="6">
+      <c r="N22" s="6">
         <v>16</v>
       </c>
-      <c r="O21">
+      <c r="O22">
         <v>2020</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B23" s="1">
         <f t="shared" si="3"/>
         <v>6.4969945355191259</v>
       </c>
-      <c r="C22">
+      <c r="C23">
         <v>23779</v>
       </c>
-      <c r="D22">
+      <c r="D23">
         <v>3660</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E23" t="s">
         <v>84</v>
       </c>
-      <c r="F22" t="s">
-        <v>64</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="F23" t="s">
+        <v>64</v>
+      </c>
+      <c r="G23" t="s">
         <v>67</v>
       </c>
-      <c r="H22">
-        <v>64</v>
-      </c>
-      <c r="I22">
+      <c r="H23">
+        <v>64</v>
+      </c>
+      <c r="I23">
         <v>14</v>
       </c>
-      <c r="J22">
+      <c r="J23">
         <v>2015</v>
       </c>
-      <c r="K22" s="1">
-        <f>C22/D22</f>
+      <c r="K23" s="1">
+        <f t="shared" ref="K23:K28" si="4">C23/D23</f>
         <v>6.4969945355191259</v>
       </c>
-      <c r="N22" s="6">
+      <c r="N23" s="6">
         <v>24</v>
       </c>
-      <c r="O22">
+      <c r="O23">
         <v>2020</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B24" s="1">
         <f t="shared" si="3"/>
         <v>7.2350710900473931</v>
       </c>
-      <c r="C23">
+      <c r="C24">
         <v>30532</v>
       </c>
-      <c r="D23">
+      <c r="D24">
         <v>4220</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E24" t="s">
         <v>85</v>
       </c>
-      <c r="F23" t="s">
-        <v>64</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="F24" t="s">
+        <v>64</v>
+      </c>
+      <c r="G24" t="s">
         <v>68</v>
       </c>
-      <c r="H23">
-        <v>64</v>
-      </c>
-      <c r="I23">
+      <c r="H24">
+        <v>64</v>
+      </c>
+      <c r="I24">
         <v>14</v>
-      </c>
-      <c r="J23">
-        <v>2020</v>
-      </c>
-      <c r="K23" s="1">
-        <f>C23/D23</f>
-        <v>7.2350710900473931</v>
-      </c>
-      <c r="N23" s="6">
-        <v>48</v>
-      </c>
-      <c r="O23">
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>103</v>
-      </c>
-      <c r="B24" s="1">
-        <f>C24/D24</f>
-        <v>7.6503125000000001</v>
-      </c>
-      <c r="C24">
-        <v>24481</v>
-      </c>
-      <c r="D24">
-        <v>3200</v>
-      </c>
-      <c r="E24" t="s">
-        <v>104</v>
-      </c>
-      <c r="F24" t="s">
-        <v>105</v>
-      </c>
-      <c r="G24" t="s">
-        <v>111</v>
-      </c>
-      <c r="H24">
-        <v>64</v>
-      </c>
-      <c r="I24">
-        <v>7</v>
       </c>
       <c r="J24">
         <v>2020</v>
       </c>
       <c r="K24" s="1">
-        <f>C24/D24</f>
+        <f t="shared" si="4"/>
+        <v>7.2350710900473931</v>
+      </c>
+      <c r="N24" s="6">
+        <v>48</v>
+      </c>
+      <c r="O24">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" s="1">
+        <f>C25/D25</f>
         <v>7.6503125000000001</v>
       </c>
-      <c r="N24" s="6">
+      <c r="C25">
+        <v>24481</v>
+      </c>
+      <c r="D25">
+        <v>3200</v>
+      </c>
+      <c r="E25" t="s">
+        <v>104</v>
+      </c>
+      <c r="F25" t="s">
+        <v>105</v>
+      </c>
+      <c r="G25" t="s">
+        <v>111</v>
+      </c>
+      <c r="H25">
+        <v>64</v>
+      </c>
+      <c r="I25">
+        <v>7</v>
+      </c>
+      <c r="J25">
+        <v>2020</v>
+      </c>
+      <c r="K25" s="1">
+        <f t="shared" si="4"/>
+        <v>7.6503125000000001</v>
+      </c>
+      <c r="N25" s="6">
         <v>8</v>
       </c>
-      <c r="O24" s="3">
+      <c r="O25" s="3">
         <v>2026</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>73</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B26" s="1">
         <f t="shared" si="3"/>
         <v>8.4960869565217383</v>
       </c>
-      <c r="C25">
+      <c r="C26">
         <v>39082</v>
       </c>
-      <c r="D25">
+      <c r="D26">
         <v>4600</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E26" t="s">
         <v>74</v>
       </c>
-      <c r="F25" t="s">
-        <v>64</v>
-      </c>
-      <c r="G25" t="s">
+      <c r="F26" t="s">
+        <v>64</v>
+      </c>
+      <c r="G26" t="s">
         <v>75</v>
       </c>
-      <c r="H25">
-        <v>64</v>
-      </c>
-      <c r="I25">
+      <c r="H26">
+        <v>64</v>
+      </c>
+      <c r="I26">
         <v>7</v>
       </c>
-      <c r="J25">
+      <c r="J26">
         <v>2023</v>
       </c>
-      <c r="K25" s="1">
-        <f>C25/D25</f>
+      <c r="K26" s="1">
+        <f t="shared" si="4"/>
         <v>8.4960869565217383</v>
       </c>
-      <c r="N25" s="6">
-        <v>64</v>
-      </c>
-      <c r="O25">
+      <c r="N26" s="6">
+        <v>64</v>
+      </c>
+      <c r="O26">
         <v>2024</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="1">
-        <f t="shared" ref="B26" si="4">C26/D26</f>
+      <c r="B27" s="1">
+        <f t="shared" ref="B27" si="5">C27/D27</f>
         <v>9.9118750000000002</v>
       </c>
-      <c r="C26">
+      <c r="C27">
         <v>31718</v>
       </c>
-      <c r="D26">
+      <c r="D27">
         <v>3200</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E27" t="s">
         <v>72</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F27" t="s">
         <v>71</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G27" t="s">
         <v>70</v>
       </c>
-      <c r="H26">
-        <v>64</v>
-      </c>
-      <c r="I26">
+      <c r="H27">
+        <v>64</v>
+      </c>
+      <c r="I27">
         <v>5</v>
       </c>
-      <c r="J26">
+      <c r="J27">
         <v>2020</v>
       </c>
-      <c r="K26" s="1">
-        <f>C26/D26</f>
+      <c r="K27" s="1">
+        <f t="shared" si="4"/>
         <v>9.9118750000000002</v>
       </c>
-      <c r="N26" s="6">
+      <c r="N27" s="6">
         <v>16</v>
       </c>
-      <c r="O26" s="3">
+      <c r="O27" s="3">
         <v>2023</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>107</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B28" s="1">
         <f t="shared" si="3"/>
         <v>10.320560747663551</v>
       </c>
-      <c r="C27">
+      <c r="C28">
         <v>33129</v>
       </c>
-      <c r="D27">
+      <c r="D28">
         <v>3210</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E28" t="s">
         <v>110</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F28" t="s">
         <v>108</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G28" t="s">
         <v>109</v>
       </c>
-      <c r="H27">
-        <v>64</v>
-      </c>
-      <c r="I27">
+      <c r="H28">
+        <v>64</v>
+      </c>
+      <c r="I28">
         <v>4</v>
       </c>
-      <c r="J27">
+      <c r="J28">
         <v>2024</v>
       </c>
-      <c r="K27" s="1">
-        <f>C27/D27</f>
+      <c r="K28" s="1">
+        <f t="shared" si="4"/>
         <v>10.320560747663551</v>
       </c>
-      <c r="M27" s="4" t="s">
+      <c r="M28" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="N27" s="6">
+      <c r="N28" s="6">
         <v>8</v>
       </c>
-      <c r="O27" s="3">
+      <c r="O28" s="3">
         <v>2026</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="B29" s="1">
-        <f>C29/D29</f>
+      <c r="B30" s="1">
+        <f>C30/D30</f>
         <v>10.320560747663551</v>
       </c>
-      <c r="C29">
+      <c r="C30">
         <v>33129</v>
       </c>
-      <c r="D29">
+      <c r="D30">
         <v>3210</v>
       </c>
-      <c r="K29" s="1">
-        <f>C29/D29</f>
+      <c r="K30" s="1">
+        <f>C30/D30</f>
         <v>10.320560747663551</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="2"/>
-      <c r="F33" t="s">
+      <c r="B34" s="2"/>
+      <c r="F34" t="s">
         <v>98</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A33" r:id="rId1" xr:uid="{1533EFA7-4865-4211-9D32-F2745D021C3D}"/>
+    <hyperlink ref="A34" r:id="rId1" xr:uid="{1533EFA7-4865-4211-9D32-F2745D021C3D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
Updated graphs and values
</commit_message>
<xml_diff>
--- a/CoreMark/CoreMark.xlsx
+++ b/CoreMark/CoreMark.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\archive\github\benchmark\CoreMark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11653733-D395-4442-A518-D3FFA44B9818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DA9E8E8-D7DC-4737-BD4B-5697C6489810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6795" yWindow="1395" windowWidth="19995" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28800" yWindow="75" windowWidth="19140" windowHeight="14730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="143">
   <si>
     <t>CoreMark Values</t>
   </si>
@@ -375,9 +375,6 @@
     <t>Kyro 585</t>
   </si>
   <si>
-    <t>Qualcomm Atheros QCA956X</t>
-  </si>
-  <si>
     <t>TP-Link Archer C7</t>
   </si>
   <si>
@@ -385,13 +382,97 @@
   </si>
   <si>
     <t>MIPS 74Kc V5.0</t>
+  </si>
+  <si>
+    <t>i5-2520M</t>
+  </si>
+  <si>
+    <t>Elitebook hp8460p</t>
+  </si>
+  <si>
+    <t>Sandy Bridge</t>
+  </si>
+  <si>
+    <t>Nehalem</t>
+  </si>
+  <si>
+    <t>Skylake</t>
+  </si>
+  <si>
+    <t>Comet Lake</t>
+  </si>
+  <si>
+    <t>Core Gen 1</t>
+  </si>
+  <si>
+    <t>Core Gen 2</t>
+  </si>
+  <si>
+    <t>Core Gen 3</t>
+  </si>
+  <si>
+    <t>Core Gen 6</t>
+  </si>
+  <si>
+    <t>Core Gen 10</t>
+  </si>
+  <si>
+    <t>Atheros QCA956X</t>
+  </si>
+  <si>
+    <t>Qualcomm</t>
+  </si>
+  <si>
+    <t>like Raspberry Pi 2</t>
+  </si>
+  <si>
+    <t>plus some AMX instr.</t>
+  </si>
+  <si>
+    <t>297 with 200 MHz</t>
+  </si>
+  <si>
+    <t>Apple M1</t>
+  </si>
+  <si>
+    <t>ESP32-C3</t>
+  </si>
+  <si>
+    <t>note3</t>
+  </si>
+  <si>
+    <t>HP Z600</t>
+  </si>
+  <si>
+    <t>Thinkpad X230</t>
+  </si>
+  <si>
+    <t>zBook 15 G3</t>
+  </si>
+  <si>
+    <t>Xigmatek Gemini</t>
+  </si>
+  <si>
+    <t>HP mini 400 G9</t>
+  </si>
+  <si>
+    <t>Macbook Air</t>
+  </si>
+  <si>
+    <t>Raptor Lake</t>
+  </si>
+  <si>
+    <t>Firestorm/Icestorm</t>
+  </si>
+  <si>
+    <t>kB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -415,8 +496,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -450,6 +550,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -487,7 +611,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -517,7 +641,58 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -886,34 +1061,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D838E1AF-0657-4DA5-A1B8-069399C72A73}">
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="4.42578125" customWidth="1"/>
     <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.85546875" customWidth="1"/>
-    <col min="14" max="14" width="5.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" customWidth="1"/>
+    <col min="14" max="14" width="8" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="N2" s="6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="H1" s="29"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H2" s="29"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
@@ -954,13 +1130,16 @@
         <v>69</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O3" s="7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P3" s="27" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>5</v>
       </c>
@@ -975,13 +1154,13 @@
         <v>16</v>
       </c>
       <c r="E4" s="14"/>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="39" t="s">
         <v>57</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="H4" s="14">
+      <c r="H4" s="30">
         <v>8</v>
       </c>
       <c r="I4" s="14"/>
@@ -994,17 +1173,20 @@
       </c>
       <c r="L4" s="14"/>
       <c r="M4" s="14"/>
-      <c r="N4" s="16"/>
+      <c r="N4" s="16" t="s">
+        <v>142</v>
+      </c>
       <c r="O4" s="14">
         <v>2020</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P4" s="14"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1">
-        <f t="shared" ref="B5:B20" si="0">C5/D5</f>
+        <f t="shared" ref="B5:B19" si="0">C5/D5</f>
         <v>1.125</v>
       </c>
       <c r="C5">
@@ -1013,13 +1195,13 @@
       <c r="D5">
         <v>72</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="36" t="s">
         <v>50</v>
       </c>
       <c r="G5" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="31">
         <v>32</v>
       </c>
       <c r="J5">
@@ -1029,11 +1211,18 @@
         <f>C5/D5</f>
         <v>1.125</v>
       </c>
+      <c r="L5">
+        <v>1.905</v>
+      </c>
+      <c r="N5" s="33">
+        <v>20</v>
+      </c>
       <c r="O5">
         <v>2020</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P5" s="22"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1047,13 +1236,13 @@
       <c r="D6">
         <v>84</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="36" t="s">
         <v>50</v>
       </c>
       <c r="G6" t="s">
         <v>52</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="31">
         <v>32</v>
       </c>
       <c r="J6">
@@ -1063,14 +1252,21 @@
         <f t="shared" ref="K6:K15" si="1">C6/D6</f>
         <v>1.7857142857142858</v>
       </c>
+      <c r="L6">
+        <v>3.42</v>
+      </c>
       <c r="M6" s="4" t="s">
         <v>53</v>
       </c>
+      <c r="N6" s="33">
+        <v>64</v>
+      </c>
       <c r="O6">
         <v>2020</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P6" s="22"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1084,13 +1280,13 @@
       <c r="D7">
         <v>100</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="36" t="s">
         <v>50</v>
       </c>
       <c r="G7" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="19">
+      <c r="H7" s="31">
         <v>32</v>
       </c>
       <c r="J7">
@@ -1100,14 +1296,21 @@
         <f t="shared" si="1"/>
         <v>1.72</v>
       </c>
+      <c r="L7">
+        <v>3.42</v>
+      </c>
       <c r="M7" s="4" t="s">
         <v>53</v>
       </c>
+      <c r="N7" s="33">
+        <v>128</v>
+      </c>
       <c r="O7">
         <v>2020</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P7" s="22"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>37</v>
       </c>
@@ -1122,15 +1325,15 @@
         <v>133</v>
       </c>
       <c r="E8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" s="36" t="s">
         <v>54</v>
       </c>
       <c r="G8" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="19">
+      <c r="H8" s="31">
         <v>32</v>
       </c>
       <c r="J8">
@@ -1140,14 +1343,16 @@
         <f t="shared" si="1"/>
         <v>1.481203007518797</v>
       </c>
-      <c r="N8" s="6">
-        <v>0.2</v>
+      <c r="M8" s="22"/>
+      <c r="N8" s="33">
+        <v>264</v>
       </c>
       <c r="O8" s="3">
         <v>2023</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P8" s="22"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>42</v>
       </c>
@@ -1164,13 +1369,13 @@
       <c r="E9" t="s">
         <v>56</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="38" t="s">
         <v>86</v>
       </c>
       <c r="G9" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="31">
         <v>32</v>
       </c>
       <c r="J9">
@@ -1180,14 +1385,18 @@
         <f t="shared" si="1"/>
         <v>1.9</v>
       </c>
-      <c r="M9" t="s">
-        <v>87</v>
+      <c r="M9" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="N9" s="33">
+        <v>400</v>
       </c>
       <c r="O9" s="3">
         <v>2023</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P9" s="22"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1201,13 +1410,13 @@
       <c r="D10">
         <v>160</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="40" t="s">
         <v>81</v>
       </c>
       <c r="G10" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="31">
         <v>32</v>
       </c>
       <c r="J10">
@@ -1217,14 +1426,18 @@
         <f t="shared" si="1"/>
         <v>2.1937500000000001</v>
       </c>
-      <c r="N10" s="6">
-        <v>0.25</v>
+      <c r="L10">
+        <v>4.1399999999999997</v>
+      </c>
+      <c r="N10" s="33">
+        <v>520</v>
       </c>
       <c r="O10">
         <v>2020</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P10" s="22"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1238,13 +1451,13 @@
       <c r="D11">
         <v>160</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="40" t="s">
         <v>81</v>
       </c>
       <c r="G11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="31">
         <v>32</v>
       </c>
       <c r="J11">
@@ -1254,14 +1467,15 @@
         <f t="shared" si="1"/>
         <v>2.2562500000000001</v>
       </c>
-      <c r="N11" s="6">
-        <v>0.25</v>
+      <c r="N11" s="33">
+        <v>520</v>
       </c>
       <c r="O11" s="3">
         <v>2023</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P11" s="22"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -1275,13 +1489,13 @@
       <c r="D12">
         <v>160</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="40" t="s">
         <v>81</v>
       </c>
       <c r="G12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="31">
         <v>32</v>
       </c>
       <c r="J12">
@@ -1291,14 +1505,15 @@
         <f t="shared" si="1"/>
         <v>2.34375</v>
       </c>
-      <c r="N12" s="6">
-        <v>0.25</v>
+      <c r="N12" s="33">
+        <v>520</v>
       </c>
       <c r="O12" s="3">
         <v>2023</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P12" s="22"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -1312,13 +1527,13 @@
       <c r="D13">
         <v>240</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="40" t="s">
         <v>81</v>
       </c>
       <c r="G13" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="19">
+      <c r="H13" s="31">
         <v>32</v>
       </c>
       <c r="J13">
@@ -1331,14 +1546,15 @@
       <c r="M13" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="N13" s="6">
-        <v>0.25</v>
+      <c r="N13" s="33">
+        <v>520</v>
       </c>
       <c r="O13" s="3">
         <v>2023</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P13" s="22"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>10</v>
       </c>
@@ -1352,13 +1568,13 @@
       <c r="D14">
         <v>700</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="36" t="s">
         <v>60</v>
       </c>
       <c r="G14" t="s">
         <v>59</v>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="31">
         <v>32</v>
       </c>
       <c r="J14">
@@ -1368,16 +1584,20 @@
         <f t="shared" si="1"/>
         <v>2.2485714285714287</v>
       </c>
-      <c r="N14" s="6">
-        <v>0.5</v>
+      <c r="L14">
+        <v>2.42</v>
+      </c>
+      <c r="N14" s="33">
+        <v>512000</v>
       </c>
       <c r="O14">
         <v>2020</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P14" s="22"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B15" s="1">
         <v>2.65</v>
@@ -1389,15 +1609,15 @@
         <v>775</v>
       </c>
       <c r="E15" t="s">
-        <v>112</v>
-      </c>
-      <c r="F15" t="s">
-        <v>115</v>
+        <v>126</v>
+      </c>
+      <c r="F15" s="38" t="s">
+        <v>114</v>
       </c>
       <c r="G15" t="s">
-        <v>114</v>
-      </c>
-      <c r="H15" s="19">
+        <v>113</v>
+      </c>
+      <c r="H15" s="31">
         <v>32</v>
       </c>
       <c r="J15">
@@ -1407,11 +1627,18 @@
         <f t="shared" si="1"/>
         <v>2.649032258064516</v>
       </c>
+      <c r="M15" t="s">
+        <v>127</v>
+      </c>
+      <c r="N15" s="33">
+        <v>128000</v>
+      </c>
       <c r="O15" s="3">
         <v>2026</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P15" s="22"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>88</v>
       </c>
@@ -1426,15 +1653,15 @@
         <v>1394</v>
       </c>
       <c r="E16" t="s">
-        <v>90</v>
-      </c>
-      <c r="F16" t="s">
+        <v>128</v>
+      </c>
+      <c r="F16" s="36" t="s">
         <v>92</v>
       </c>
       <c r="G16" t="s">
         <v>89</v>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="31">
         <v>32</v>
       </c>
       <c r="J16">
@@ -1444,12 +1671,13 @@
         <f>C16/D16</f>
         <v>2.8436154949784793</v>
       </c>
-      <c r="N16" s="6">
-        <v>1</v>
+      <c r="N16" s="33">
+        <v>1024000</v>
       </c>
       <c r="O16" s="3">
         <v>2025</v>
       </c>
+      <c r="P16" s="22"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
@@ -1465,16 +1693,14 @@
       <c r="D17" s="12">
         <v>1200</v>
       </c>
-      <c r="E17" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="F17" s="12" t="s">
+      <c r="E17" s="23"/>
+      <c r="F17" s="37" t="s">
         <v>62</v>
       </c>
       <c r="G17" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H17" s="12">
+      <c r="H17" s="32">
         <v>64</v>
       </c>
       <c r="I17" s="12"/>
@@ -1485,7 +1711,9 @@
         <f>C17/D17</f>
         <v>3.1666666666666665</v>
       </c>
-      <c r="L17" s="12"/>
+      <c r="L17" s="12">
+        <v>2.6</v>
+      </c>
       <c r="M17" s="12"/>
       <c r="N17" s="13">
         <v>1</v>
@@ -1493,9 +1721,7 @@
       <c r="O17" s="12">
         <v>2020</v>
       </c>
-      <c r="P17" t="s">
-        <v>98</v>
-      </c>
+      <c r="P17" s="12"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
@@ -1511,498 +1737,597 @@
       <c r="D18">
         <v>1200</v>
       </c>
-      <c r="E18" t="s">
-        <v>95</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="E18" s="24"/>
+      <c r="F18" s="36" t="s">
         <v>63</v>
       </c>
       <c r="G18" t="s">
         <v>61</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="29">
         <v>64</v>
       </c>
       <c r="J18">
         <v>2015</v>
       </c>
       <c r="K18" s="1">
-        <f t="shared" ref="K18:K22" si="2">C18/D18</f>
+        <f t="shared" ref="K18:K23" si="2">C18/D18</f>
         <v>3.2608333333333333</v>
+      </c>
+      <c r="N18" s="6">
+        <v>2</v>
       </c>
       <c r="O18">
         <v>2020</v>
       </c>
+      <c r="P18" s="22"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
-        <v>91</v>
+      <c r="A19" t="s">
+        <v>13</v>
       </c>
       <c r="B19" s="1">
         <f t="shared" si="0"/>
-        <v>5.504666666666667</v>
+        <v>4.4584967320261439</v>
       </c>
       <c r="C19">
-        <v>8257</v>
+        <v>13643</v>
       </c>
       <c r="D19">
-        <v>1500</v>
-      </c>
-      <c r="E19" t="s">
-        <v>94</v>
-      </c>
-      <c r="F19" t="s">
-        <v>63</v>
+        <v>3060</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="F19" s="34" t="s">
+        <v>64</v>
       </c>
       <c r="G19" t="s">
-        <v>93</v>
-      </c>
-      <c r="H19">
-        <v>64</v>
+        <v>65</v>
+      </c>
+      <c r="H19" s="29">
+        <v>64</v>
+      </c>
+      <c r="I19">
+        <v>45</v>
       </c>
       <c r="J19">
-        <v>2019</v>
+        <v>2009</v>
       </c>
       <c r="K19" s="1">
         <f t="shared" si="2"/>
-        <v>5.504666666666667</v>
+        <v>4.4584967320261439</v>
+      </c>
+      <c r="M19" t="s">
+        <v>118</v>
       </c>
       <c r="N19" s="6">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="O19">
-        <v>2025</v>
+        <v>2020</v>
+      </c>
+      <c r="P19" s="22" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="1">
-        <f t="shared" si="0"/>
-        <v>4.4584967320261439</v>
-      </c>
-      <c r="C20">
-        <v>13643</v>
-      </c>
-      <c r="D20">
-        <v>3060</v>
-      </c>
-      <c r="E20" t="s">
-        <v>83</v>
-      </c>
-      <c r="F20" t="s">
-        <v>64</v>
-      </c>
-      <c r="G20" t="s">
-        <v>65</v>
-      </c>
-      <c r="H20">
-        <v>64</v>
-      </c>
-      <c r="I20">
-        <v>45</v>
-      </c>
-      <c r="J20">
-        <v>2009</v>
+      <c r="A20" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" s="25">
+        <v>5.4</v>
+      </c>
+      <c r="C20" s="20">
+        <v>13500</v>
+      </c>
+      <c r="D20" s="20">
+        <v>2500</v>
+      </c>
+      <c r="E20" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="F20" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="H20" s="21">
+        <v>64</v>
+      </c>
+      <c r="I20" s="20">
+        <v>32</v>
+      </c>
+      <c r="J20" s="22">
+        <v>2011</v>
       </c>
       <c r="K20" s="1">
         <f t="shared" si="2"/>
-        <v>4.4584967320261439</v>
-      </c>
-      <c r="N20" s="6">
-        <v>24</v>
-      </c>
-      <c r="O20">
-        <v>2020</v>
+        <v>5.4</v>
+      </c>
+      <c r="L20" s="22"/>
+      <c r="M20" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="N20" s="21">
+        <v>16</v>
+      </c>
+      <c r="O20" s="20">
+        <v>2024</v>
+      </c>
+      <c r="P20" s="28" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="A21" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="1">
+        <f t="shared" ref="B21" si="3">C21/D21</f>
+        <v>5.504666666666667</v>
+      </c>
+      <c r="C21">
+        <v>8257</v>
+      </c>
+      <c r="D21">
+        <v>1500</v>
+      </c>
+      <c r="E21" s="24"/>
+      <c r="F21" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="G21" t="s">
+        <v>93</v>
+      </c>
+      <c r="H21" s="29">
+        <v>64</v>
+      </c>
+      <c r="I21">
+        <v>28</v>
+      </c>
+      <c r="J21">
+        <v>2019</v>
+      </c>
+      <c r="K21" s="1">
+        <f t="shared" ref="K21" si="4">C21/D21</f>
+        <v>5.504666666666667</v>
+      </c>
+      <c r="N21" s="6">
+        <v>4</v>
+      </c>
+      <c r="O21">
+        <v>2025</v>
+      </c>
+      <c r="P21" s="22"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>76</v>
       </c>
-      <c r="B21" s="1">
-        <f>C21/D21</f>
+      <c r="B22" s="1">
+        <f>C22/D22</f>
         <v>6.3620000000000001</v>
       </c>
-      <c r="C21">
+      <c r="C22">
         <v>19086</v>
       </c>
-      <c r="D21">
+      <c r="D22">
         <v>3000</v>
       </c>
-      <c r="E21" t="s">
-        <v>82</v>
-      </c>
-      <c r="F21" t="s">
-        <v>64</v>
-      </c>
-      <c r="G21" t="s">
+      <c r="E22" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="F22" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" t="s">
         <v>66</v>
       </c>
-      <c r="H21">
-        <v>64</v>
-      </c>
-      <c r="I21">
+      <c r="H22" s="29">
+        <v>64</v>
+      </c>
+      <c r="I22">
         <v>22</v>
       </c>
-      <c r="J21">
+      <c r="J22">
         <v>2013</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K22" s="1">
         <f t="shared" si="2"/>
         <v>6.3620000000000001</v>
       </c>
-      <c r="N21" s="6">
+      <c r="M22" t="s">
+        <v>66</v>
+      </c>
+      <c r="N22" s="6">
         <v>16</v>
       </c>
-      <c r="O21">
+      <c r="O22">
         <v>2024</v>
       </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="P22" s="22"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="1">
-        <f t="shared" ref="B22:B28" si="3">C22/D22</f>
+      <c r="B23" s="1">
+        <f t="shared" ref="B23:B29" si="5">C23/D23</f>
         <v>6.4378787878787875</v>
       </c>
-      <c r="C22">
+      <c r="C23">
         <v>21245</v>
       </c>
-      <c r="D22">
+      <c r="D23">
         <v>3300</v>
       </c>
-      <c r="E22" t="s">
-        <v>82</v>
-      </c>
-      <c r="F22" t="s">
-        <v>64</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="E23" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="F23" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="G23" t="s">
         <v>66</v>
       </c>
-      <c r="H22">
-        <v>64</v>
-      </c>
-      <c r="I22">
+      <c r="H23" s="29">
+        <v>64</v>
+      </c>
+      <c r="I23">
         <v>22</v>
       </c>
-      <c r="J22">
+      <c r="J23">
         <v>2012</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K23" s="1">
         <f t="shared" si="2"/>
         <v>6.4378787878787875</v>
       </c>
-      <c r="N22" s="6">
+      <c r="M23" t="s">
+        <v>66</v>
+      </c>
+      <c r="N23" s="6">
         <v>16</v>
-      </c>
-      <c r="O22">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" s="1">
-        <f t="shared" si="3"/>
-        <v>6.4969945355191259</v>
-      </c>
-      <c r="C23">
-        <v>23779</v>
-      </c>
-      <c r="D23">
-        <v>3660</v>
-      </c>
-      <c r="E23" t="s">
-        <v>84</v>
-      </c>
-      <c r="F23" t="s">
-        <v>64</v>
-      </c>
-      <c r="G23" t="s">
-        <v>67</v>
-      </c>
-      <c r="H23">
-        <v>64</v>
-      </c>
-      <c r="I23">
-        <v>14</v>
-      </c>
-      <c r="J23">
-        <v>2015</v>
-      </c>
-      <c r="K23" s="1">
-        <f t="shared" ref="K23:K28" si="4">C23/D23</f>
-        <v>6.4969945355191259</v>
-      </c>
-      <c r="N23" s="6">
-        <v>24</v>
       </c>
       <c r="O23">
         <v>2020</v>
       </c>
+      <c r="P23" s="19" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="B24" s="1">
-        <f t="shared" si="3"/>
-        <v>7.2350710900473931</v>
+        <f t="shared" si="5"/>
+        <v>6.4969945355191259</v>
       </c>
       <c r="C24">
-        <v>30532</v>
+        <v>23779</v>
       </c>
       <c r="D24">
-        <v>4220</v>
-      </c>
-      <c r="E24" t="s">
-        <v>85</v>
-      </c>
-      <c r="F24" t="s">
+        <v>3660</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="F24" s="34" t="s">
         <v>64</v>
       </c>
       <c r="G24" t="s">
-        <v>68</v>
-      </c>
-      <c r="H24">
+        <v>67</v>
+      </c>
+      <c r="H24" s="29">
         <v>64</v>
       </c>
       <c r="I24">
         <v>14</v>
       </c>
       <c r="J24">
+        <v>2015</v>
+      </c>
+      <c r="K24" s="1">
+        <f t="shared" ref="K24:K29" si="6">C24/D24</f>
+        <v>6.4969945355191259</v>
+      </c>
+      <c r="M24" t="s">
+        <v>119</v>
+      </c>
+      <c r="N24" s="6">
+        <v>24</v>
+      </c>
+      <c r="O24">
         <v>2020</v>
       </c>
-      <c r="K24" s="1">
-        <f t="shared" si="4"/>
-        <v>7.2350710900473931</v>
-      </c>
-      <c r="N24" s="6">
-        <v>48</v>
-      </c>
-      <c r="O24">
-        <v>2021</v>
+      <c r="P24" s="19" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>103</v>
+        <v>16</v>
       </c>
       <c r="B25" s="1">
-        <f>C25/D25</f>
-        <v>7.6503125000000001</v>
+        <f t="shared" si="5"/>
+        <v>7.2350710900473931</v>
       </c>
       <c r="C25">
-        <v>24481</v>
+        <v>30532</v>
       </c>
       <c r="D25">
-        <v>3200</v>
-      </c>
-      <c r="E25" t="s">
-        <v>104</v>
-      </c>
-      <c r="F25" t="s">
-        <v>105</v>
+        <v>4220</v>
+      </c>
+      <c r="E25" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="F25" s="34" t="s">
+        <v>64</v>
       </c>
       <c r="G25" t="s">
-        <v>111</v>
-      </c>
-      <c r="H25">
+        <v>68</v>
+      </c>
+      <c r="H25" s="29">
         <v>64</v>
       </c>
       <c r="I25">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J25">
         <v>2020</v>
       </c>
       <c r="K25" s="1">
-        <f t="shared" si="4"/>
-        <v>7.6503125000000001</v>
+        <f t="shared" si="6"/>
+        <v>7.2350710900473931</v>
+      </c>
+      <c r="M25" t="s">
+        <v>120</v>
       </c>
       <c r="N25" s="6">
-        <v>8</v>
-      </c>
-      <c r="O25" s="3">
-        <v>2026</v>
+        <v>48</v>
+      </c>
+      <c r="O25">
+        <v>2021</v>
+      </c>
+      <c r="P25" s="28" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="B26" s="1">
-        <f t="shared" si="3"/>
-        <v>8.4960869565217383</v>
+        <f>C26/D26</f>
+        <v>7.6503125000000001</v>
       </c>
       <c r="C26">
-        <v>39082</v>
+        <v>24481</v>
       </c>
       <c r="D26">
-        <v>4600</v>
-      </c>
-      <c r="E26" t="s">
-        <v>74</v>
-      </c>
-      <c r="F26" t="s">
-        <v>64</v>
+        <v>3200</v>
+      </c>
+      <c r="E26" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="F26" s="36" t="s">
+        <v>105</v>
       </c>
       <c r="G26" t="s">
-        <v>75</v>
-      </c>
-      <c r="H26">
+        <v>111</v>
+      </c>
+      <c r="H26" s="29">
         <v>64</v>
       </c>
       <c r="I26">
         <v>7</v>
       </c>
       <c r="J26">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="K26" s="1">
-        <f t="shared" si="4"/>
-        <v>8.4960869565217383</v>
+        <f t="shared" si="6"/>
+        <v>7.6503125000000001</v>
+      </c>
+      <c r="M26" t="s">
+        <v>104</v>
       </c>
       <c r="N26" s="6">
-        <v>64</v>
-      </c>
-      <c r="O26">
-        <v>2024</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O26" s="3">
+        <v>2026</v>
+      </c>
+      <c r="P26" s="22"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="B27" s="1">
-        <f t="shared" ref="B27" si="5">C27/D27</f>
-        <v>9.9118750000000002</v>
+        <f t="shared" si="5"/>
+        <v>8.4960869565217383</v>
       </c>
       <c r="C27">
-        <v>31718</v>
+        <v>39082</v>
       </c>
       <c r="D27">
-        <v>3200</v>
-      </c>
-      <c r="E27" t="s">
-        <v>72</v>
-      </c>
-      <c r="F27" t="s">
-        <v>71</v>
+        <v>4600</v>
+      </c>
+      <c r="E27" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="F27" s="34" t="s">
+        <v>64</v>
       </c>
       <c r="G27" t="s">
-        <v>70</v>
-      </c>
-      <c r="H27">
+        <v>75</v>
+      </c>
+      <c r="H27" s="29">
         <v>64</v>
       </c>
       <c r="I27">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J27">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="K27" s="1">
-        <f t="shared" si="4"/>
-        <v>9.9118750000000002</v>
+        <f t="shared" si="6"/>
+        <v>8.4960869565217383</v>
+      </c>
+      <c r="M27" t="s">
+        <v>140</v>
       </c>
       <c r="N27" s="6">
-        <v>16</v>
-      </c>
-      <c r="O27" s="3">
-        <v>2023</v>
+        <v>64</v>
+      </c>
+      <c r="O27">
+        <v>2024</v>
+      </c>
+      <c r="P27" s="19" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="1">
+        <f t="shared" ref="B28" si="7">C28/D28</f>
+        <v>9.9118750000000002</v>
+      </c>
+      <c r="C28">
+        <v>31718</v>
+      </c>
+      <c r="D28">
+        <v>3200</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="F28" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="G28" t="s">
+        <v>70</v>
+      </c>
+      <c r="H28" s="29">
+        <v>64</v>
+      </c>
+      <c r="I28">
+        <v>5</v>
+      </c>
+      <c r="J28">
+        <v>2020</v>
+      </c>
+      <c r="K28" s="1">
+        <f t="shared" si="6"/>
+        <v>9.9118750000000002</v>
+      </c>
+      <c r="M28" t="s">
+        <v>141</v>
+      </c>
+      <c r="N28" s="6">
+        <v>16</v>
+      </c>
+      <c r="O28" s="3">
+        <v>2023</v>
+      </c>
+      <c r="P28" s="19" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>107</v>
       </c>
-      <c r="B28" s="1">
-        <f t="shared" si="3"/>
+      <c r="B29" s="1">
+        <f t="shared" si="5"/>
         <v>10.320560747663551</v>
       </c>
-      <c r="C28">
+      <c r="C29">
         <v>33129</v>
       </c>
-      <c r="D28">
+      <c r="D29">
         <v>3210</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E29" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F29" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G29" t="s">
         <v>109</v>
       </c>
-      <c r="H28">
-        <v>64</v>
-      </c>
-      <c r="I28">
+      <c r="H29" s="29">
+        <v>64</v>
+      </c>
+      <c r="I29">
         <v>4</v>
       </c>
-      <c r="J28">
+      <c r="J29">
         <v>2024</v>
       </c>
-      <c r="K28" s="1">
-        <f t="shared" si="4"/>
+      <c r="K29" s="1">
+        <f t="shared" si="6"/>
         <v>10.320560747663551</v>
       </c>
-      <c r="M28" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="N28" s="6">
+      <c r="M29" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="N29" s="6">
         <v>8</v>
       </c>
-      <c r="O28" s="3">
+      <c r="O29" s="3">
         <v>2026</v>
       </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" s="17" t="s">
+      <c r="P29" s="22"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="B30" s="1">
-        <f>C30/D30</f>
+      <c r="B31" s="1">
+        <f>C31/D31</f>
         <v>10.320560747663551</v>
       </c>
-      <c r="C30">
+      <c r="C31">
         <v>33129</v>
       </c>
-      <c r="D30">
+      <c r="D31">
         <v>3210</v>
       </c>
-      <c r="K30" s="1">
-        <f>C30/D30</f>
+      <c r="K31" s="1">
+        <f>C31/D31</f>
         <v>10.320560747663551</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B34" s="2"/>
-      <c r="F34" t="s">
+      <c r="B35" s="2"/>
+      <c r="F35" t="s">
         <v>98</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A34" r:id="rId1" xr:uid="{1533EFA7-4865-4211-9D32-F2745D021C3D}"/>
+    <hyperlink ref="A35" r:id="rId1" xr:uid="{1533EFA7-4865-4211-9D32-F2745D021C3D}"/>
+    <hyperlink ref="M9" r:id="rId2" location="riscvcpu" display="https://www.espressif.com/sites/default/files/documentation/esp32-c3_technical_reference_manual_en.pdf - riscvcpu" xr:uid="{66F7B36A-23BF-4B96-9B61-331676444F22}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Include Galaxy Note 8
</commit_message>
<xml_diff>
--- a/CoreMark/CoreMark.xlsx
+++ b/CoreMark/CoreMark.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\archive\github\benchmark\CoreMark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DA9E8E8-D7DC-4737-BD4B-5697C6489810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4626615D-3B8A-4DB7-A255-E2815A1CD02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="75" windowWidth="19140" windowHeight="14730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15945" yWindow="1350" windowWidth="22215" windowHeight="14730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="4" r:id="rId1"/>
@@ -36,8 +36,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="146">
   <si>
     <t>CoreMark Values</t>
   </si>
@@ -466,6 +488,15 @@
   </si>
   <si>
     <t>kB</t>
+  </si>
+  <si>
+    <t>Galaxy Note 8</t>
+  </si>
+  <si>
+    <t>Exynos 8895</t>
+  </si>
+  <si>
+    <t>Exynos M2</t>
   </si>
 </sst>
 </file>
@@ -1061,7 +1092,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D838E1AF-0657-4DA5-A1B8-069399C72A73}">
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -1077,6 +1108,7 @@
     <col min="12" max="12" width="8.85546875" customWidth="1"/>
     <col min="13" max="13" width="14.42578125" customWidth="1"/>
     <col min="14" max="14" width="8" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1186,7 +1218,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="1">
-        <f t="shared" ref="B5:B19" si="0">C5/D5</f>
+        <f t="shared" ref="B5:B20" si="0">C5/D5</f>
         <v>1.125</v>
       </c>
       <c r="C5">
@@ -1751,7 +1783,7 @@
         <v>2015</v>
       </c>
       <c r="K18" s="1">
-        <f t="shared" ref="K18:K23" si="2">C18/D18</f>
+        <f t="shared" ref="K18:K24" si="2">C18/D18</f>
         <v>3.2608333333333333</v>
       </c>
       <c r="N18" s="6">
@@ -1812,518 +1844,565 @@
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="B20" s="25">
-        <v>5.4</v>
-      </c>
-      <c r="C20" s="20">
-        <v>13500</v>
-      </c>
-      <c r="D20" s="20">
-        <v>2500</v>
+      <c r="A20" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B20" s="1">
+        <f t="shared" si="0"/>
+        <v>4.7329004329004327</v>
+      </c>
+      <c r="C20">
+        <v>10933</v>
+      </c>
+      <c r="D20">
+        <v>2310</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>122</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="G20" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="H20" s="21">
-        <v>64</v>
-      </c>
-      <c r="I20" s="20">
-        <v>32</v>
-      </c>
-      <c r="J20" s="22">
-        <v>2011</v>
+        <v>144</v>
+      </c>
+      <c r="F20" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" t="s">
+        <v>145</v>
+      </c>
+      <c r="H20" s="29">
+        <v>64</v>
+      </c>
+      <c r="I20">
+        <v>10</v>
+      </c>
+      <c r="J20">
+        <v>2017</v>
       </c>
       <c r="K20" s="1">
         <f t="shared" si="2"/>
+        <v>4.7329004329004327</v>
+      </c>
+      <c r="N20" s="6">
+        <v>6</v>
+      </c>
+      <c r="O20" s="3">
+        <v>2026</v>
+      </c>
+      <c r="P20" s="22" cm="1">
+        <f t="array" aca="1" ref="P20" ca="1">+P20:BA20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B21" s="25">
         <v>5.4</v>
       </c>
-      <c r="L20" s="22"/>
-      <c r="M20" s="19" t="s">
+      <c r="C21" s="20">
+        <v>13500</v>
+      </c>
+      <c r="D21" s="20">
+        <v>2500</v>
+      </c>
+      <c r="E21" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="F21" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="H21" s="21">
+        <v>64</v>
+      </c>
+      <c r="I21" s="20">
+        <v>32</v>
+      </c>
+      <c r="J21" s="22">
+        <v>2011</v>
+      </c>
+      <c r="K21" s="1">
+        <f t="shared" si="2"/>
+        <v>5.4</v>
+      </c>
+      <c r="L21" s="22"/>
+      <c r="M21" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="N20" s="21">
+      <c r="N21" s="21">
         <v>16</v>
       </c>
-      <c r="O20" s="20">
+      <c r="O21" s="20">
         <v>2024</v>
       </c>
-      <c r="P20" s="28" t="s">
+      <c r="P21" s="28" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="9" t="s">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="B21" s="1">
-        <f t="shared" ref="B21" si="3">C21/D21</f>
+      <c r="B22" s="1">
+        <f t="shared" ref="B22" si="3">C22/D22</f>
         <v>5.504666666666667</v>
       </c>
-      <c r="C21">
+      <c r="C22">
         <v>8257</v>
       </c>
-      <c r="D21">
+      <c r="D22">
         <v>1500</v>
       </c>
-      <c r="E21" s="24"/>
-      <c r="F21" s="36" t="s">
+      <c r="E22" s="24"/>
+      <c r="F22" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G22" t="s">
         <v>93</v>
       </c>
-      <c r="H21" s="29">
-        <v>64</v>
-      </c>
-      <c r="I21">
+      <c r="H22" s="29">
+        <v>64</v>
+      </c>
+      <c r="I22">
         <v>28</v>
       </c>
-      <c r="J21">
+      <c r="J22">
         <v>2019</v>
       </c>
-      <c r="K21" s="1">
-        <f t="shared" ref="K21" si="4">C21/D21</f>
+      <c r="K22" s="1">
+        <f t="shared" ref="K22" si="4">C22/D22</f>
         <v>5.504666666666667</v>
       </c>
-      <c r="N21" s="6">
+      <c r="N22" s="6">
         <v>4</v>
       </c>
-      <c r="O21">
+      <c r="O22">
         <v>2025</v>
       </c>
-      <c r="P21" s="22"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="P22" s="22"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="1">
-        <f>C22/D22</f>
+      <c r="B23" s="1">
+        <f>C23/D23</f>
         <v>6.3620000000000001</v>
       </c>
-      <c r="C22">
+      <c r="C23">
         <v>19086</v>
       </c>
-      <c r="D22">
+      <c r="D23">
         <v>3000</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E23" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="F22" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="F23" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="G23" t="s">
         <v>66</v>
       </c>
-      <c r="H22" s="29">
-        <v>64</v>
-      </c>
-      <c r="I22">
+      <c r="H23" s="29">
+        <v>64</v>
+      </c>
+      <c r="I23">
         <v>22</v>
       </c>
-      <c r="J22">
+      <c r="J23">
         <v>2013</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K23" s="1">
         <f t="shared" si="2"/>
         <v>6.3620000000000001</v>
       </c>
-      <c r="M22" t="s">
+      <c r="M23" t="s">
         <v>66</v>
       </c>
-      <c r="N22" s="6">
+      <c r="N23" s="6">
         <v>16</v>
       </c>
-      <c r="O22">
+      <c r="O23">
         <v>2024</v>
       </c>
-      <c r="P22" s="22"/>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="P23" s="22"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="1">
-        <f t="shared" ref="B23:B29" si="5">C23/D23</f>
+      <c r="B24" s="1">
+        <f t="shared" ref="B24:B30" si="5">C24/D24</f>
         <v>6.4378787878787875</v>
       </c>
-      <c r="C23">
+      <c r="C24">
         <v>21245</v>
       </c>
-      <c r="D23">
+      <c r="D24">
         <v>3300</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E24" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="F23" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="F24" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="G24" t="s">
         <v>66</v>
       </c>
-      <c r="H23" s="29">
-        <v>64</v>
-      </c>
-      <c r="I23">
+      <c r="H24" s="29">
+        <v>64</v>
+      </c>
+      <c r="I24">
         <v>22</v>
       </c>
-      <c r="J23">
+      <c r="J24">
         <v>2012</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K24" s="1">
         <f t="shared" si="2"/>
         <v>6.4378787878787875</v>
       </c>
-      <c r="M23" t="s">
+      <c r="M24" t="s">
         <v>66</v>
       </c>
-      <c r="N23" s="6">
+      <c r="N24" s="6">
         <v>16</v>
       </c>
-      <c r="O23">
+      <c r="O24">
         <v>2020</v>
       </c>
-      <c r="P23" s="19" t="s">
+      <c r="P24" s="19" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B25" s="1">
         <f t="shared" si="5"/>
         <v>6.4969945355191259</v>
       </c>
-      <c r="C24">
+      <c r="C25">
         <v>23779</v>
       </c>
-      <c r="D24">
+      <c r="D25">
         <v>3660</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E25" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="F24" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="G24" t="s">
+      <c r="F25" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="G25" t="s">
         <v>67</v>
       </c>
-      <c r="H24" s="29">
-        <v>64</v>
-      </c>
-      <c r="I24">
+      <c r="H25" s="29">
+        <v>64</v>
+      </c>
+      <c r="I25">
         <v>14</v>
       </c>
-      <c r="J24">
+      <c r="J25">
         <v>2015</v>
       </c>
-      <c r="K24" s="1">
-        <f t="shared" ref="K24:K29" si="6">C24/D24</f>
+      <c r="K25" s="1">
+        <f t="shared" ref="K25:K30" si="6">C25/D25</f>
         <v>6.4969945355191259</v>
       </c>
-      <c r="M24" t="s">
+      <c r="M25" t="s">
         <v>119</v>
       </c>
-      <c r="N24" s="6">
+      <c r="N25" s="6">
         <v>24</v>
       </c>
-      <c r="O24">
+      <c r="O25">
         <v>2020</v>
       </c>
-      <c r="P24" s="19" t="s">
+      <c r="P25" s="19" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>16</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B26" s="1">
         <f t="shared" si="5"/>
         <v>7.2350710900473931</v>
       </c>
-      <c r="C25">
+      <c r="C26">
         <v>30532</v>
       </c>
-      <c r="D25">
+      <c r="D26">
         <v>4220</v>
       </c>
-      <c r="E25" s="24" t="s">
+      <c r="E26" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="F25" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="G25" t="s">
+      <c r="F26" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="G26" t="s">
         <v>68</v>
       </c>
-      <c r="H25" s="29">
-        <v>64</v>
-      </c>
-      <c r="I25">
+      <c r="H26" s="29">
+        <v>64</v>
+      </c>
+      <c r="I26">
         <v>14</v>
       </c>
-      <c r="J25">
+      <c r="J26">
         <v>2020</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K26" s="1">
         <f t="shared" si="6"/>
         <v>7.2350710900473931</v>
       </c>
-      <c r="M25" t="s">
+      <c r="M26" t="s">
         <v>120</v>
       </c>
-      <c r="N25" s="6">
+      <c r="N26" s="6">
         <v>48</v>
       </c>
-      <c r="O25">
+      <c r="O26">
         <v>2021</v>
       </c>
-      <c r="P25" s="28" t="s">
+      <c r="P26" s="28" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B26" s="1">
-        <f>C26/D26</f>
+      <c r="B27" s="1">
+        <f>C27/D27</f>
         <v>7.6503125000000001</v>
       </c>
-      <c r="C26">
+      <c r="C27">
         <v>24481</v>
       </c>
-      <c r="D26">
+      <c r="D27">
         <v>3200</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E27" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="F26" s="36" t="s">
+      <c r="F27" s="36" t="s">
         <v>105</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G27" t="s">
         <v>111</v>
       </c>
-      <c r="H26" s="29">
-        <v>64</v>
-      </c>
-      <c r="I26">
+      <c r="H27" s="29">
+        <v>64</v>
+      </c>
+      <c r="I27">
         <v>7</v>
       </c>
-      <c r="J26">
+      <c r="J27">
         <v>2020</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K27" s="1">
         <f t="shared" si="6"/>
         <v>7.6503125000000001</v>
       </c>
-      <c r="M26" t="s">
+      <c r="M27" t="s">
         <v>104</v>
       </c>
-      <c r="N26" s="6">
+      <c r="N27" s="6">
         <v>8</v>
       </c>
-      <c r="O26" s="3">
+      <c r="O27" s="3">
         <v>2026</v>
       </c>
-      <c r="P26" s="22"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="P27" s="22"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>73</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B28" s="1">
         <f t="shared" si="5"/>
         <v>8.4960869565217383</v>
       </c>
-      <c r="C27">
+      <c r="C28">
         <v>39082</v>
       </c>
-      <c r="D27">
+      <c r="D28">
         <v>4600</v>
       </c>
-      <c r="E27" s="24" t="s">
+      <c r="E28" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="F27" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="G27" t="s">
+      <c r="F28" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="G28" t="s">
         <v>75</v>
       </c>
-      <c r="H27" s="29">
-        <v>64</v>
-      </c>
-      <c r="I27">
+      <c r="H28" s="29">
+        <v>64</v>
+      </c>
+      <c r="I28">
         <v>7</v>
       </c>
-      <c r="J27">
+      <c r="J28">
         <v>2023</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K28" s="1">
         <f t="shared" si="6"/>
         <v>8.4960869565217383</v>
       </c>
-      <c r="M27" t="s">
+      <c r="M28" t="s">
         <v>140</v>
       </c>
-      <c r="N27" s="6">
-        <v>64</v>
-      </c>
-      <c r="O27">
+      <c r="N28" s="6">
+        <v>64</v>
+      </c>
+      <c r="O28">
         <v>2024</v>
       </c>
-      <c r="P27" s="19" t="s">
+      <c r="P28" s="19" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>131</v>
       </c>
-      <c r="B28" s="1">
-        <f t="shared" ref="B28" si="7">C28/D28</f>
+      <c r="B29" s="1">
+        <f t="shared" ref="B29" si="7">C29/D29</f>
         <v>9.9118750000000002</v>
       </c>
-      <c r="C28">
+      <c r="C29">
         <v>31718</v>
       </c>
-      <c r="D28">
+      <c r="D29">
         <v>3200</v>
       </c>
-      <c r="E28" s="24" t="s">
+      <c r="E29" s="24" t="s">
         <v>129</v>
       </c>
-      <c r="F28" s="36" t="s">
+      <c r="F29" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G29" t="s">
         <v>70</v>
       </c>
-      <c r="H28" s="29">
-        <v>64</v>
-      </c>
-      <c r="I28">
+      <c r="H29" s="29">
+        <v>64</v>
+      </c>
+      <c r="I29">
         <v>5</v>
       </c>
-      <c r="J28">
+      <c r="J29">
         <v>2020</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K29" s="1">
         <f t="shared" si="6"/>
         <v>9.9118750000000002</v>
       </c>
-      <c r="M28" t="s">
+      <c r="M29" t="s">
         <v>141</v>
       </c>
-      <c r="N28" s="6">
+      <c r="N29" s="6">
         <v>16</v>
       </c>
-      <c r="O28" s="3">
+      <c r="O29" s="3">
         <v>2023</v>
       </c>
-      <c r="P28" s="19" t="s">
+      <c r="P29" s="19" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B30" s="1">
         <f t="shared" si="5"/>
         <v>10.320560747663551</v>
       </c>
-      <c r="C29">
+      <c r="C30">
         <v>33129</v>
       </c>
-      <c r="D29">
+      <c r="D30">
         <v>3210</v>
       </c>
-      <c r="E29" s="24" t="s">
+      <c r="E30" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="F29" s="36" t="s">
+      <c r="F30" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G30" t="s">
         <v>109</v>
       </c>
-      <c r="H29" s="29">
-        <v>64</v>
-      </c>
-      <c r="I29">
+      <c r="H30" s="29">
+        <v>64</v>
+      </c>
+      <c r="I30">
         <v>4</v>
       </c>
-      <c r="J29">
+      <c r="J30">
         <v>2024</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K30" s="1">
         <f t="shared" si="6"/>
         <v>10.320560747663551</v>
       </c>
-      <c r="M29" s="4" t="s">
+      <c r="M30" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="N29" s="6">
+      <c r="N30" s="6">
         <v>8</v>
       </c>
-      <c r="O29" s="3">
+      <c r="O30" s="3">
         <v>2026</v>
       </c>
-      <c r="P29" s="22"/>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A31" s="17" t="s">
+      <c r="P30" s="22"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="B31" s="1">
-        <f>C31/D31</f>
-        <v>10.320560747663551</v>
-      </c>
-      <c r="C31">
-        <v>33129</v>
-      </c>
-      <c r="D31">
-        <v>3210</v>
-      </c>
-      <c r="K31" s="1">
-        <f>C31/D31</f>
-        <v>10.320560747663551</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="B32" s="1">
+        <f>C32/D32</f>
+        <v>4.7329004329004327</v>
+      </c>
+      <c r="C32">
+        <v>10933</v>
+      </c>
+      <c r="D32">
+        <v>2310</v>
+      </c>
+      <c r="K32" s="1">
+        <f>C32/D32</f>
+        <v>4.7329004329004327</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="2"/>
-      <c r="F35" t="s">
+      <c r="B36" s="2"/>
+      <c r="F36" t="s">
         <v>98</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A35" r:id="rId1" xr:uid="{1533EFA7-4865-4211-9D32-F2745D021C3D}"/>
+    <hyperlink ref="A36" r:id="rId1" xr:uid="{1533EFA7-4865-4211-9D32-F2745D021C3D}"/>
     <hyperlink ref="M9" r:id="rId2" location="riscvcpu" display="https://www.espressif.com/sites/default/files/documentation/esp32-c3_technical_reference_manual_en.pdf - riscvcpu" xr:uid="{66F7B36A-23BF-4B96-9B61-331676444F22}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>